<commit_message>
fixing issues related to ui export and reports left
</commit_message>
<xml_diff>
--- a/gayatri_invoice/gayatriapp/main/media/Reports/stock_report.xlsx
+++ b/gayatri_invoice/gayatriapp/main/media/Reports/stock_report.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -631,6 +631,62 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>800</v>
+      </c>
+      <c r="J6" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" t="n">
+        <v>651</v>
+      </c>
+      <c r="N6" t="n">
+        <v>653</v>
+      </c>
+      <c r="O6" t="n">
+        <v>456</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>213321</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>5644</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>4656545</t>
         </is>
       </c>
     </row>
@@ -647,7 +703,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -663,6 +719,62 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>800</v>
+      </c>
+      <c r="J7" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>649</v>
+      </c>
+      <c r="N7" t="n">
+        <v>650</v>
+      </c>
+      <c r="O7" t="n">
+        <v>456</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>213321</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>5644</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>4656545</t>
         </is>
       </c>
     </row>
@@ -679,7 +791,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -695,6 +807,62 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>800</v>
+      </c>
+      <c r="J8" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="n">
+        <v>646</v>
+      </c>
+      <c r="N8" t="n">
+        <v>648</v>
+      </c>
+      <c r="O8" t="n">
+        <v>456</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>213321</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>5644</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>4656545</t>
         </is>
       </c>
     </row>
@@ -711,7 +879,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -727,6 +895,62 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>120</v>
+      </c>
+      <c r="J9" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" t="n">
+        <v>100</v>
+      </c>
+      <c r="M9" t="n">
+        <v>545</v>
+      </c>
+      <c r="N9" t="n">
+        <v>645</v>
+      </c>
+      <c r="O9" t="n">
+        <v>123</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -743,7 +967,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -759,6 +983,62 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>120</v>
+      </c>
+      <c r="J10" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M10" t="n">
+        <v>545</v>
+      </c>
+      <c r="N10" t="n">
+        <v>645</v>
+      </c>
+      <c r="O10" t="n">
+        <v>123</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -775,7 +1055,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -791,6 +1071,62 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>120</v>
+      </c>
+      <c r="J11" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>100</v>
+      </c>
+      <c r="M11" t="n">
+        <v>545</v>
+      </c>
+      <c r="N11" t="n">
+        <v>645</v>
+      </c>
+      <c r="O11" t="n">
+        <v>123</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -807,7 +1143,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BUNDLE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -823,6 +1159,62 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>539</v>
+      </c>
+      <c r="N12" t="n">
+        <v>544</v>
+      </c>
+      <c r="O12" t="n">
+        <v>123</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>231213</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -839,7 +1231,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BULK</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -855,6 +1247,62 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>12</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12</v>
+      </c>
+      <c r="L13" t="n">
+        <v>103</v>
+      </c>
+      <c r="M13" t="n">
+        <v>435</v>
+      </c>
+      <c r="N13" t="n">
+        <v>538</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>231213</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>132231</t>
         </is>
       </c>
     </row>
@@ -871,7 +1319,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BULK</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -887,6 +1335,62 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>12</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>12</v>
+      </c>
+      <c r="L14" t="n">
+        <v>100</v>
+      </c>
+      <c r="M14" t="n">
+        <v>334</v>
+      </c>
+      <c r="N14" t="n">
+        <v>434</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>231213</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>132231</t>
         </is>
       </c>
     </row>
@@ -903,7 +1407,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>BULK</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -919,6 +1423,62 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>12</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>12</v>
+      </c>
+      <c r="L15" t="n">
+        <v>123</v>
+      </c>
+      <c r="M15" t="n">
+        <v>210</v>
+      </c>
+      <c r="N15" t="n">
+        <v>333</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>231213</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>132231</t>
         </is>
       </c>
     </row>

</xml_diff>